<commit_message>
UPDATE codigo e Inputs
</commit_message>
<xml_diff>
--- a/Inputs/Inputs.xlsx
+++ b/Inputs/Inputs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Codigos\HU_SCS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Codigos\HU_SCS\Inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9989D8CD-1FC5-41ED-ABB9-5A6E1611DB9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AD2228B-8509-46A4-B2DA-D8E8D7EEA264}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info Cuencas" sheetId="1" r:id="rId1"/>
@@ -334,8 +334,8 @@
     <xdr:to>
       <xdr:col>23</xdr:col>
       <xdr:colOff>59055</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>76199</xdr:rowOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -350,8 +350,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15889605" y="380999"/>
-          <a:ext cx="2819400" cy="2028825"/>
+          <a:off x="15916275" y="380999"/>
+          <a:ext cx="2819400" cy="647701"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -406,42 +406,6 @@
               </a:solidFill>
             </a:rPr>
           </a:br>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="es-CL" sz="1100" b="1">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Nota para el codigo: si no se ingresa ningun valor de tiempo de concentración adoptado,</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> detener el código y enviar mensaje de alerta. Si se ingresa un valor inferior a 10 minutos, enviar un mensaje de alerta y preguntar si se quiere continuar con este valor.</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-            </a:rPr>
-          </a:br>
           <a:endParaRPr lang="en-US" sz="1100" b="1">
             <a:solidFill>
               <a:srgbClr val="FF0000"/>
@@ -457,112 +421,6 @@
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>11430</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>129540</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>15240</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>161925</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="TextBox 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{43548CE5-F1D6-48C7-A32F-E341AF0F50C6}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6831330" y="1558290"/>
-          <a:ext cx="4347210" cy="575310"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="38100" cmpd="sng">
-          <a:solidFill>
-            <a:srgbClr val="FF0000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr marL="0" indent="0"/>
-          <a:r>
-            <a:rPr lang="es-CL" sz="1100" b="1">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Nota para el codigo: si no se ingresa ningun delta D adoptado, detener el codigo</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> y enviar mensaje de alerta.</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-          </a:br>
-          <a:endParaRPr lang="es-CL" sz="1100" b="1">
-            <a:solidFill>
-              <a:srgbClr val="FF0000"/>
-            </a:solidFill>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>9</xdr:col>
@@ -684,8 +542,8 @@
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>80010</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>100966</xdr:rowOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -700,8 +558,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2438400" y="180975"/>
-          <a:ext cx="4347210" cy="1548766"/>
+          <a:off x="2438400" y="182880"/>
+          <a:ext cx="4347210" cy="2270760"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -743,7 +601,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>En esta pestaña se deben agregar las precipitaciones máximas en 24 horas para los períodos de retorno que se quieren analizar.</a:t>
+            <a:t>En esta pestaña se deben agregar las precipitaciones máximas para los períodos de retorno que se quieren analizar.</a:t>
           </a:r>
           <a:br>
             <a:rPr lang="es-CL" sz="1100" b="1">
@@ -796,38 +654,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t> todas las precipitaciones máximas en 24 horas que se ingresen.</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="es-CL" sz="1100" b="1">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-          </a:br>
-          <a:br>
-            <a:rPr lang="es-CL" sz="1100" b="1">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="es-CL" sz="1100" b="1">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Nota para el codigo: si no se ingresa ninguna Pp Max, detener el codigo y enviar mensaje de alerta.</a:t>
+            <a:t> todas las precipitaciones máximas que se ingresen.</a:t>
           </a:r>
           <a:br>
             <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
@@ -840,81 +667,19 @@
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
           </a:br>
-          <a:endParaRPr lang="es-CL" sz="1100" b="1">
-            <a:solidFill>
-              <a:srgbClr val="FF0000"/>
-            </a:solidFill>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>81915</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>97156</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="TextBox 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9ACE1258-6722-4F98-9FA6-6BA08DCA017C}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="7315200" y="180975"/>
-          <a:ext cx="4349115" cy="1544956"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="38100" cmpd="sng">
-          <a:solidFill>
-            <a:srgbClr val="FF0000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr marL="0" indent="0"/>
+          <a:br>
+            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
           <a:r>
-            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
+            <a:rPr lang="es-CL" sz="1100" b="1" u="sng" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="FF0000"/>
               </a:solidFill>
@@ -923,7 +688,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Nota para el codigo:</a:t>
+            <a:t>Importante:</a:t>
           </a:r>
           <a:br>
             <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
@@ -946,12 +711,12 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Preguntar a copilot si habría problemas con que en "T" se rellenen dos períodos de retorno iguales, o si habría problemas con poner un string acá (como por ejemplo "T=2-CC")</a:t>
+            <a:t>No se pueden agregar periodos de retorno duplicados.</a:t>
           </a:r>
           <a:br>
             <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:srgbClr val="FF0000"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -959,6 +724,41 @@
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
           </a:br>
+          <a:r>
+            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Si se pueden agregar cadenas de texto en el periodo de retorno del tipo "2-CC".</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Los valores de Pp Max deben ser numéricos.</a:t>
+          </a:r>
           <a:endParaRPr lang="es-CL" sz="1100" b="1">
             <a:solidFill>
               <a:srgbClr val="FF0000"/>
@@ -987,8 +787,8 @@
     <xdr:to>
       <xdr:col>9</xdr:col>
       <xdr:colOff>360045</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>104776</xdr:rowOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1003,8 +803,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2438400" y="180976"/>
-          <a:ext cx="3408045" cy="1733550"/>
+          <a:off x="2438400" y="182881"/>
+          <a:ext cx="3408045" cy="2034539"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1122,102 +922,7 @@
             </a:rPr>
           </a:br>
           <a:r>
-            <a:rPr lang="es-CL" sz="1100" b="1">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Nota para el codigo: si no se ingresa ningún CD, detener</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> el codigo y enviar mensaje de alerta.</a:t>
-          </a:r>
-          <a:endParaRPr lang="es-CL" sz="1100" b="1">
-            <a:solidFill>
-              <a:srgbClr val="FF0000"/>
-            </a:solidFill>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>83820</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>93346</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="TextBox 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3C2A0A9D-A96A-4588-9008-7CD268890179}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6096000" y="180975"/>
-          <a:ext cx="4351020" cy="1541146"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="38100" cmpd="sng">
-          <a:solidFill>
-            <a:srgbClr val="FF0000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr marL="0" indent="0"/>
-          <a:r>
-            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
+            <a:rPr lang="es-CL" sz="1100" b="1" u="sng" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="FF0000"/>
               </a:solidFill>
@@ -1226,7 +931,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Nota para el codigo:</a:t>
+            <a:t>Importante:</a:t>
           </a:r>
           <a:br>
             <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
@@ -1249,14 +954,59 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Preguntar a copilot si habría problemas con que en "Horas" se rellenen dos duraciones iguales, o si habría problemas con poner un string o un número que no sea entero (aunque esto ultimo no se si se dé en hidrología).</a:t>
+            <a:t>No se pueden agregar duraciones duplicadas.</a:t>
           </a:r>
           <a:br>
             <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:srgbClr val="FF0000"/>
               </a:solidFill>
               <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>No se pueden agregar cadenas de texto como duración.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="es-CL" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Los valores de CD deben ser numéricos.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="es-CL" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
               <a:latin typeface="+mn-lt"/>
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
@@ -25039,6 +24789,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="40414187-dd76-4ef8-b04f-ccddae734140" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="63768118-86e2-4829-8a12-b72c47658d02">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CCB1C2B958A07241A317F5A881DFD30C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ec29f518eb9a62149baea9c73f5411cd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="63768118-86e2-4829-8a12-b72c47658d02" xmlns:ns3="40414187-dd76-4ef8-b04f-ccddae734140" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="29f6242226419d82ce7554acb1ee2c31" ns2:_="" ns3:_="">
     <xsd:import namespace="63768118-86e2-4829-8a12-b72c47658d02"/>
@@ -25293,27 +25063,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A4DA3E6-B8B6-48A6-81EC-CAAD4DEE707B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="40414187-dd76-4ef8-b04f-ccddae734140"/>
+    <ds:schemaRef ds:uri="63768118-86e2-4829-8a12-b72c47658d02"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="40414187-dd76-4ef8-b04f-ccddae734140" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="63768118-86e2-4829-8a12-b72c47658d02">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26BC43C4-0DE4-4398-8C07-F13A3433226F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{124384BF-B442-43EF-BEBD-26F0C03197F3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -25330,23 +25099,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26BC43C4-0DE4-4398-8C07-F13A3433226F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A4DA3E6-B8B6-48A6-81EC-CAAD4DEE707B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="40414187-dd76-4ef8-b04f-ccddae734140"/>
-    <ds:schemaRef ds:uri="63768118-86e2-4829-8a12-b72c47658d02"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>